<commit_message>
feat: adicionar parcelamento em lançamentos a prazo
</commit_message>
<xml_diff>
--- a/fornecedores_ficticios.xlsx
+++ b/fornecedores_ficticios.xlsx
@@ -921,6 +921,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1246,7 +1250,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K51"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="28.59765625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="23.796875" bestFit="1" customWidth="1"/>
@@ -1261,7 +1265,7 @@
     <col min="11" max="11" width="6.69921875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1296,7 +1300,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -1331,7 +1335,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>21</v>
       </c>
@@ -1366,7 +1370,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>29</v>
       </c>
@@ -1401,7 +1405,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>35</v>
       </c>
@@ -1436,7 +1440,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>42</v>
       </c>
@@ -1471,7 +1475,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>50</v>
       </c>
@@ -1506,7 +1510,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>56</v>
       </c>
@@ -1541,7 +1545,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>61</v>
       </c>
@@ -1576,7 +1580,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>66</v>
       </c>
@@ -1611,7 +1615,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>73</v>
       </c>
@@ -1646,7 +1650,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>79</v>
       </c>
@@ -1681,7 +1685,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>84</v>
       </c>
@@ -1716,7 +1720,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>91</v>
       </c>
@@ -1751,7 +1755,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>96</v>
       </c>
@@ -1786,7 +1790,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>101</v>
       </c>
@@ -1821,7 +1825,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>107</v>
       </c>
@@ -1856,7 +1860,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>112</v>
       </c>
@@ -1891,7 +1895,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>117</v>
       </c>
@@ -1926,7 +1930,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="20" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>122</v>
       </c>
@@ -1961,7 +1965,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="21" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>127</v>
       </c>
@@ -1996,7 +2000,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="22" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>132</v>
       </c>
@@ -2031,7 +2035,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="23" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>137</v>
       </c>
@@ -2066,7 +2070,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="24" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>142</v>
       </c>
@@ -2101,7 +2105,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="25" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>147</v>
       </c>
@@ -2136,7 +2140,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="26" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>152</v>
       </c>
@@ -2171,7 +2175,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="27" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>157</v>
       </c>
@@ -2206,7 +2210,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="28" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>162</v>
       </c>
@@ -2241,7 +2245,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="29" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>167</v>
       </c>
@@ -2276,7 +2280,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="30" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>172</v>
       </c>
@@ -2311,7 +2315,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="31" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>178</v>
       </c>
@@ -2346,7 +2350,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="32" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>183</v>
       </c>
@@ -2381,7 +2385,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="33" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>188</v>
       </c>
@@ -2416,7 +2420,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="34" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>193</v>
       </c>
@@ -2451,7 +2455,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="35" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>198</v>
       </c>
@@ -2486,7 +2490,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="36" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>203</v>
       </c>
@@ -2521,7 +2525,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="37" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>208</v>
       </c>
@@ -2556,7 +2560,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="38" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>213</v>
       </c>
@@ -2591,7 +2595,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="39" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>218</v>
       </c>
@@ -2626,7 +2630,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="40" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>223</v>
       </c>
@@ -2661,7 +2665,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="41" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>228</v>
       </c>
@@ -2696,7 +2700,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="42" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>233</v>
       </c>
@@ -2731,7 +2735,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="43" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>238</v>
       </c>
@@ -2766,7 +2770,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="44" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>243</v>
       </c>
@@ -2801,7 +2805,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="45" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>248</v>
       </c>
@@ -2836,7 +2840,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="46" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>253</v>
       </c>
@@ -2871,7 +2875,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="47" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>258</v>
       </c>
@@ -2906,7 +2910,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="48" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>263</v>
       </c>
@@ -2941,7 +2945,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="49" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>268</v>
       </c>
@@ -2976,7 +2980,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="50" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>273</v>
       </c>
@@ -3011,7 +3015,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="51" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>278</v>
       </c>
@@ -3049,7 +3053,7 @@
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:K51" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:K13 A15:K51 B14:K14" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>